<commit_message>
Back up current vault before course audit consolidation
</commit_message>
<xml_diff>
--- a/_vault_setup/01_md_convert/korean_yt_md_convert.xlsx
+++ b/_vault_setup/01_md_convert/korean_yt_md_convert.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vault\Koreanwithji_vault\_vault_setup\01_md_convert\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\vault\koreanwithji_vault\_vault_setup\01_md_convert\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C69BCB2D-98EE-4462-80B1-4DB834B53803}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{579B7F7C-9B6A-4156-B608-5B2EAB3ECABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="7500" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="70">
   <si>
     <t>Ji 레벨</t>
   </si>
@@ -226,6 +226,21 @@
   </si>
   <si>
     <t>https://youtu.be/_cIyKLjMgW4</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>How Korean works</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>hanafromkorea</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>https://youtu.be/JwgvBB2GTto</t>
+  </si>
+  <si>
+    <t>The fundamental cultural differences between Eastern and Western mindsets</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -589,7 +604,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -774,34 +789,28 @@
     <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="6" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="7" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="4" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="3" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="7" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="7">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1125,22 +1134,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.7"/>
+  <dimension ref="A1:K14"/>
+  <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="7.34765625" style="60" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.34765625" style="60" customWidth="1"/>
-    <col min="4" max="4" width="9.09765625" style="60" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.09765625" style="60" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.59765625" style="60" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="7.33203125" style="60" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" style="60" customWidth="1"/>
+    <col min="4" max="4" width="9.08203125" style="60" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15" style="60" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.58203125" style="60" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.75" style="60" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="113.25" style="60" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.09765625" style="60" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.34765625" style="60" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.08203125" style="60" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.33203125" style="60" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="9.25" style="60" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="1" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1184,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="132" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="2" spans="1:11" ht="132" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="23">
         <v>1</v>
       </c>
@@ -1203,14 +1212,14 @@
       <c r="I2" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K2" s="63" t="s">
+      <c r="J2" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K2" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="49.5" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="3" spans="1:11" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -1235,17 +1244,17 @@
       <c r="H3" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="64" t="s">
+      <c r="I3" s="63" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K3" s="63" t="s">
+      <c r="J3" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="4" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="9">
         <v>1</v>
       </c>
@@ -1273,14 +1282,14 @@
       <c r="I4" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="63" t="s">
+      <c r="J4" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K4" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="49.5" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="5" spans="1:11" ht="49.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="17">
         <v>1</v>
       </c>
@@ -1308,14 +1317,14 @@
       <c r="I5" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="J5" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K5" s="63" t="s">
+      <c r="J5" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K5" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="6" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="29">
         <v>1</v>
       </c>
@@ -1325,7 +1334,7 @@
       <c r="C6" s="30" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="65" t="s">
+      <c r="D6" s="64" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="31" t="s">
@@ -1340,17 +1349,17 @@
       <c r="H6" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="I6" s="66" t="s">
+      <c r="I6" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="J6" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K6" s="63" t="s">
+      <c r="J6" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K6" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="7" spans="1:11" ht="33" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="35">
         <v>5</v>
       </c>
@@ -1369,23 +1378,23 @@
       <c r="F7" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="67" t="s">
+      <c r="G7" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="H7" s="67" t="s">
+      <c r="H7" s="66" t="s">
         <v>41</v>
       </c>
-      <c r="I7" s="67" t="s">
+      <c r="I7" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="J7" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K7" s="63" t="s">
+      <c r="J7" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K7" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="8" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="39">
         <v>6</v>
       </c>
@@ -1413,14 +1422,14 @@
       <c r="I8" s="44" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K8" s="63" t="s">
+      <c r="J8" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.7">
+    <row r="9" spans="1:11" ht="66" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="45">
         <v>8</v>
       </c>
@@ -1445,17 +1454,17 @@
       <c r="H9" s="51" t="s">
         <v>50</v>
       </c>
-      <c r="I9" s="68" t="s">
+      <c r="I9" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K9" s="63" t="s">
+      <c r="J9" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:11" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A10" s="52">
         <v>8</v>
       </c>
@@ -1481,18 +1490,18 @@
       <c r="I10" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="J10" s="63" t="s">
-        <v>18</v>
-      </c>
-      <c r="K10" s="63" t="s">
+      <c r="J10" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="62" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="16.8" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A11" s="69">
+    <row r="11" spans="1:11" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A11">
         <v>3</v>
       </c>
-      <c r="B11" s="69">
+      <c r="B11">
         <v>12</v>
       </c>
       <c r="C11" s="61" t="s">
@@ -1507,28 +1516,28 @@
       <c r="F11" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="G11" s="69"/>
-      <c r="H11" s="70" t="s">
+      <c r="G11"/>
+      <c r="H11" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="I11" s="69" t="s">
+      <c r="I11" t="s">
         <v>54</v>
       </c>
-      <c r="J11" s="63" t="s">
+      <c r="J11" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="K11" s="63" t="s">
+      <c r="K11" s="62" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="49.8" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A12" s="69">
+    <row r="12" spans="1:11" ht="51.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A12">
         <v>6</v>
       </c>
-      <c r="B12" s="69">
+      <c r="B12">
         <v>9</v>
       </c>
-      <c r="C12" s="70" t="s">
+      <c r="C12" s="68" t="s">
         <v>64</v>
       </c>
       <c r="D12" s="55" t="s">
@@ -1540,28 +1549,28 @@
       <c r="F12" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="G12" s="69"/>
-      <c r="H12" s="69" t="s">
+      <c r="G12"/>
+      <c r="H12" t="s">
         <v>61</v>
       </c>
-      <c r="I12" s="69" t="s">
+      <c r="I12" t="s">
         <v>60</v>
       </c>
       <c r="J12" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="K12" s="63" t="s">
+      <c r="K12" s="62" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="16.8" thickBot="1" x14ac:dyDescent="0.75">
-      <c r="A13" s="69">
+    <row r="13" spans="1:11" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A13">
         <v>11</v>
       </c>
-      <c r="B13" s="69">
+      <c r="B13">
         <v>5</v>
       </c>
-      <c r="C13" s="70" t="s">
+      <c r="C13" s="68" t="s">
         <v>63</v>
       </c>
       <c r="D13" s="55" t="s">
@@ -1573,18 +1582,42 @@
       <c r="F13" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="G13" s="69"/>
-      <c r="H13" s="69" t="s">
+      <c r="G13"/>
+      <c r="H13" t="s">
         <v>62</v>
       </c>
-      <c r="I13" s="71" t="s">
+      <c r="I13" s="69" t="s">
         <v>65</v>
       </c>
       <c r="J13" s="62" t="s">
         <v>55</v>
       </c>
-      <c r="K13" s="63" t="s">
+      <c r="K13" s="62" t="s">
         <v>56</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="17.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A14" s="60">
+        <v>1</v>
+      </c>
+      <c r="B14" s="60">
+        <v>1</v>
+      </c>
+      <c r="C14" s="60" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="F14" s="32"/>
+      <c r="H14" s="60" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="60" t="s">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>